<commit_message>
chore: refresh Excel results template from latest sample run
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/ket_qua_template.xlsx
+++ b/excel/ket_qua_template.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-07-14T14:57:46</t>
+          <t>2026-07-14T15:59:37</t>
         </is>
       </c>
     </row>

</xml_diff>